<commit_message>
chore(report-cards): clearer gradebook placeholders + lualatex guidance
Rename the starter-gradebook roster to obvious placeholders
(John/Jane/Jamie Doe; scores unchanged) so the sample reads as dummy
data. Add the `% !TeX program = lualatex` magic comment to the
report-card template and document in the README why every report-card
doc needs it (a pdflatex build dies with "\gradebook requires LuaLaTeX").

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Report Cards/gradebook.xlsx
+++ b/Report Cards/gradebook.xlsx
@@ -101,7 +101,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sample Student</t>
+          <t xml:space="preserve">John Doe</t>
         </is>
       </c>
       <c r="B2">
@@ -156,7 +156,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jordan Lee</t>
+          <t xml:space="preserve">Jane Doe</t>
         </is>
       </c>
       <c r="B3">
@@ -211,7 +211,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alex Kim</t>
+          <t xml:space="preserve">Jamie Doe</t>
         </is>
       </c>
       <c r="B4">
@@ -505,7 +505,7 @@
     <row r="2">
       <c r="A2" t="str">
         <f>Roster!A2</f>
-        <v>Sample Student</v>
+        <v>John Doe</v>
       </c>
       <c r="B2">
         <v>15</v>
@@ -682,7 +682,7 @@
     <row r="3">
       <c r="A3" t="str">
         <f>Roster!A3</f>
-        <v>Jordan Lee</v>
+        <v>Jane Doe</v>
       </c>
       <c r="B3">
         <v>15</v>
@@ -859,7 +859,7 @@
     <row r="4">
       <c r="A4" t="str">
         <f>Roster!A4</f>
-        <v>Alex Kim</v>
+        <v>Jamie Doe</v>
       </c>
       <c r="B4">
         <v>15</v>

</xml_diff>